<commit_message>
fix(xlsx/chart): warn on misscaled referenceLine and wrong label position
Two silent foot-guns in referenceLine: (1) a numeric value > 1 on a
percent-stacked chart where the val axis is 0-1, causing Excel to
auto-scale the axis (e.g. to 5000%) and visually compress the real
bars to a sliver on the left; (2) the format has no width field, so
'50:FF0000:1.5:dash' puts '1.5' into the label slot and surfaces as
the legend text.

Add non-blocking warnings for both: a range check when
IsPercentStackedChart(plotArea) && refValue > 1.0, and a heuristic
that fires when parts.Length==4 && parts[2] parses as a number &&
parts[3] is a known dash style. Both go to stderr; behavior is
unchanged so the only cost to a legitimate numeric label is one
ignorable line on stderr.

Also fix charts-basic example: referenceLine=50:FF0000:1.5:dash ->
0.5:FF0000:Target:dash, with a comment documenting the 0-1 axis
and the lack of a width field. Regenerate charts-basic.xlsx.
</commit_message>
<xml_diff>
--- a/examples/excel/charts-basic.xlsx
+++ b/examples/excel/charts-basic.xlsx
@@ -3,13 +3,13 @@
 <x:workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
     <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="rId1"/>
-    <x:sheet name="1-Column Charts" sheetId="2" r:id="R814498b81b644840"/>
-    <x:sheet name="2-Bar Charts" sheetId="3" r:id="Rf4d9d7ed04d9436c"/>
-    <x:sheet name="3-Line Charts" sheetId="4" r:id="Rf7609b9eda7f49bd"/>
-    <x:sheet name="4-Area Charts" sheetId="5" r:id="R19b01bc7be3c47fc"/>
-    <x:sheet name="5-Styling" sheetId="6" r:id="Rb375c6bc6ec4484b"/>
-    <x:sheet name="6-Layout" sheetId="7" r:id="R01f066a9198e4e59"/>
-    <x:sheet name="7-Effects" sheetId="8" r:id="R23769b43821a4939"/>
+    <x:sheet name="1-Column Charts" sheetId="2" r:id="R560a4bf398d94f01"/>
+    <x:sheet name="2-Bar Charts" sheetId="3" r:id="Ra307cbd6b4f4441c"/>
+    <x:sheet name="3-Line Charts" sheetId="4" r:id="Re3598e0b3cdf47fa"/>
+    <x:sheet name="4-Area Charts" sheetId="5" r:id="Rc8e69b068a2c46d3"/>
+    <x:sheet name="5-Styling" sheetId="6" r:id="Rfb14b7252fc84210"/>
+    <x:sheet name="6-Layout" sheetId="7" r:id="Rd437f303bdbc441e"/>
+    <x:sheet name="7-Effects" sheetId="8" r:id="R0837b779f65a41f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9420,7 +9420,7 @@
           <c:idx val="4"/>
           <c:order val="4"/>
           <c:tx>
-            <c:v>1.5</c:v>
+            <c:v>Target</c:v>
           </c:tx>
           <c:spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="19050">
@@ -9438,40 +9438,40 @@
               <c:formatCode>General</c:formatCode>
               <c:ptCount val="12"/>
               <c:pt idx="0">
-                <c:v>50</c:v>
+                <c:v>0.5</c:v>
               </c:pt>
               <c:pt idx="1">
-                <c:v>50</c:v>
+                <c:v>0.5</c:v>
               </c:pt>
               <c:pt idx="2">
-                <c:v>50</c:v>
+                <c:v>0.5</c:v>
               </c:pt>
               <c:pt idx="3">
-                <c:v>50</c:v>
+                <c:v>0.5</c:v>
               </c:pt>
               <c:pt idx="4">
-                <c:v>50</c:v>
+                <c:v>0.5</c:v>
               </c:pt>
               <c:pt idx="5">
-                <c:v>50</c:v>
+                <c:v>0.5</c:v>
               </c:pt>
               <c:pt idx="6">
-                <c:v>50</c:v>
+                <c:v>0.5</c:v>
               </c:pt>
               <c:pt idx="7">
-                <c:v>50</c:v>
+                <c:v>0.5</c:v>
               </c:pt>
               <c:pt idx="8">
-                <c:v>50</c:v>
+                <c:v>0.5</c:v>
               </c:pt>
               <c:pt idx="9">
-                <c:v>50</c:v>
+                <c:v>0.5</c:v>
               </c:pt>
               <c:pt idx="10">
-                <c:v>50</c:v>
+                <c:v>0.5</c:v>
               </c:pt>
               <c:pt idx="11">
-                <c:v>50</c:v>
+                <c:v>0.5</c:v>
               </c:pt>
             </c:numLit>
           </c:val>
@@ -10157,7 +10157,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6d53490f6d404a3d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R24718cc0980d4fc4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10187,7 +10187,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R91e784ae75d3422f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R26bebb52a8c84a5b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10217,7 +10217,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb4f5287ccf6041d7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R432dd9cf996a4477"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10247,7 +10247,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rcbe573f9381c4acd"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7764e1f6101d4a04"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10282,7 +10282,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9a6b48ac0f3f48d1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R247838841eb243ce"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10312,7 +10312,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R24fb5da4030b4bf1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re2d1bdff31e14704"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10342,7 +10342,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc9b237d8a55244f1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R00480fe234004afe"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10372,7 +10372,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf980951eeae14c9d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rddcf743be72448c7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10407,7 +10407,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8ee6147aa3164ced"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R21f3bd03a26f456b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10437,7 +10437,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9f5448b63a0648a5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7a3080d6813d4c03"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10467,7 +10467,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbff5b9774eb44581"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7e8ef4350d474a4b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10497,7 +10497,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R83d92fe3b2fc42f3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R65048789872c451f"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10532,7 +10532,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7b949c5d76d24aca"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R458a7b96f2894d9c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10562,7 +10562,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re7f35015c8304b0f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R08349980ebf04e90"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10592,7 +10592,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd2677761202e4cd1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R93598b57b04b4af7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10622,7 +10622,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R88813e1ff59749b1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R25023aaf1f3c4bd3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10657,7 +10657,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R52275c3162b64fe7"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbf4413b997034260"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10687,7 +10687,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5ce2d32c68544e1a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rbbeb739ec15a4f06"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10717,7 +10717,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1ae197f5e93547d4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rab6081858cac4d3c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10747,7 +10747,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R58571bc23c544750"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re0f15ccdde594f94"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10782,7 +10782,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0ea799e2e9ee4f80"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R729d8afe59bb4881"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10812,7 +10812,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3cd2000395de4edf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7347994c558345fd"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10842,7 +10842,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R24271b43031e45d0"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R667668fa10bf47d8"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10872,7 +10872,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf96c637b9bac4a5a"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R52c96cea30594025"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10907,7 +10907,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9c3b0a405b804d92"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra1d9756de84e41f6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10937,7 +10937,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdad5b2e519f340ee"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5a8b6d30e71e4327"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10967,7 +10967,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd657072be46e4c94"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2b5f4a480d184b1c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -10997,7 +10997,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdf8d2b0299334de0"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R60655219932349b6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -11237,48 +11237,48 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recbd9e04451142ee"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15e25689d885457f"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c57a4e1235c4fbd"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e9f1930d6b942a5"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ad906b4b29d4c6a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1752ad416534669"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6da8894a672f4f5d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a796ab3d4104728"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra76ca9878c514746"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c4c2c9aed3e49ec"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84f89ca568164ec0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0dbedbcc516f4826"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetData/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R64409c8068d240bb"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbdfab560920e4fe7"/>
 </x:worksheet>
 </file>
</xml_diff>